<commit_message>
progress: 37 village workbooks (rw-rtx-3070 2026-10-09T22:20:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Kizhmuthalambedu_13.357765_80.134189.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Kizhmuthalambedu_13.357765_80.134189.xlsx
@@ -1454,6 +1454,11 @@
           <t>340</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2A3, 2A4, 2B, 2C, 2D1, 2D2, 2D3, 2D4, 2D5, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1461,6 +1466,11 @@
           <t>341</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>10, 11, 1A, 1B, 1C, 1D, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1468,6 +1478,11 @@
           <t>342</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>10A1, 10A2, 10A3, 10A4, 10A5, 10B, 10C1, 10C2, 10C3, 10C4, 11A1, 11A2, 11A3, 11B, 12, 13, 14, 15, 16, 17, 18, 19, 1A1, 1A1B, 1A2, 1B1, 1B2, 2, 20, 21, 22, 23, 24, 25, 3, 4A, 4B, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1475,6 +1490,11 @@
           <t>343</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 10, 11A1, 11A2, 11B1, 11B2, 12, 13, 2, 3, 4, 5, 6A, 6B, 6C, 6D, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1482,6 +1502,11 @@
           <t>344</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1489,6 +1514,11 @@
           <t>345</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B1, 6B2, 7A1, 7A2, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1496,6 +1526,11 @@
           <t>346</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3, 4, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1503,6 +1538,11 @@
           <t>347</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 3A, 3B, 3C, 4, 5A, 5B, 5C, 5D</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1510,6 +1550,11 @@
           <t>348</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1517,6 +1562,11 @@
           <t>349</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B1, 1B2, 2A1, 2A2, 2A3, 2A4, 3A1, 3A2, 3B1</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1524,6 +1574,11 @@
           <t>350</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B, 3A1, 3A2, 3B, 3C, 4A1, 4A2, 4B1, 4B2, 4C1, 4C2</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1531,6 +1586,11 @@
           <t>351</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 3, 4A, 4B, 4C</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1538,6 +1598,11 @@
           <t>352</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1545,6 +1610,11 @@
           <t>353</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2, 2B1, 2B2, 2C, 3A, 3B, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1552,6 +1622,11 @@
           <t>354</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1559,6 +1634,11 @@
           <t>355</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2A, 2B, 2C, 3, 4A, 4B, 5A, 5B, 6, 7A1A1A, 7A1B, 7A2, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1566,6 +1646,11 @@
           <t>356</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14A, 14B, 14C, 2, 3, 4, 5, 6A, 6B, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1573,6 +1658,11 @@
           <t>357</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1580,6 +1670,11 @@
           <t>358</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 1A, 1B1, 1B2, 1C, 1D, 1E, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1587,6 +1682,11 @@
           <t>359</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 19, 2A, 2B, 3, 4, 5, 6, 7A, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1594,6 +1694,11 @@
           <t>360</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1, 10, 11A1, 11A2, 11B, 12, 13, 14, 15A, 15B, 16A, 16B, 17, 2, 3, 4, 5A, 5B, 6, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1601,6 +1706,11 @@
           <t>361</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1608,6 +1718,11 @@
           <t>362</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3A, 3B, 4A, 4B, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1615,6 +1730,11 @@
           <t>363</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12A, 12B1, 12B2, 13, 14, 2A, 2B, 3, 4, 5, 6, 7A, 7B1, 7B2, 7B3, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1622,6 +1742,11 @@
           <t>364</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 1A, 1B1, 1B2, 1C, 1D, 1E, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 7C, 7D, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1629,6 +1754,11 @@
           <t>365</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 16, 17A, 17B, 17C, 18A, 18B, 19, 2, 20, 21, 22, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1636,6 +1766,11 @@
           <t>366</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1643,6 +1778,11 @@
           <t>367</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5A, 5B, 5C, 5D, 6A, 6B, 6C, 6D, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1650,6 +1790,11 @@
           <t>368</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1, 10A1, 10A2, 10A3, 10B, 11, 12, 13, 14, 15A, 15B, 16, 17, 18, 19, 2, 20, 21A, 21B, 22, 23, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1657,6 +1802,11 @@
           <t>369</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 1A1, 1A2, 1B, 2A, 2B, 2C, 3, 4A, 4B, 4C, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1664,6 +1814,11 @@
           <t>370</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13, 14, 15, 1A, 1B, 1C, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1671,6 +1826,11 @@
           <t>371</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3A, 3B, 4, 5, 6, 7, 8A, 8B, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1678,6 +1838,11 @@
           <t>372</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3A1, 3A2, 3B, 3C, 3D, 3E, 4A, 4B, 5A, 5B, 6A, 6B, 7A, 7B, 8</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1685,6 +1850,11 @@
           <t>373</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12, 13, 14A, 14B, 15A, 15B, 1A, 1B, 2A, 2B, 3, 4, 5A, 5B, 6, 7, 8A, 8B, 8C, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1692,6 +1862,11 @@
           <t>374</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6A1A, 6A1B, 6A1C, 6A2, 6B, 6C1, 6C2</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1699,6 +1874,11 @@
           <t>375</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5, 6A, 6B1, 6B2, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1706,6 +1886,11 @@
           <t>376</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3A, 3B, 4A, 4B, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1713,6 +1898,11 @@
           <t>377</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 3, 4A, 4B, 5, 6A1, 6A2, 6B1, 6B2, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1720,6 +1910,11 @@
           <t>378</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A1, 14A2, 14A3, 14B, 15, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1727,6 +1922,11 @@
           <t>379</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1734,6 +1934,11 @@
           <t>380</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 1A, 1B, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1741,6 +1946,11 @@
           <t>381</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B, 4C, 5, 6, 7, 8, 9A, 9B, 9C</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1748,6 +1958,11 @@
           <t>382</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1755,6 +1970,11 @@
           <t>383</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1762,6 +1982,11 @@
           <t>384</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1769,6 +1994,11 @@
           <t>385</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3, 4, 5, 6, 7, 8A1, 8A2, 8B1, 8B2</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1776,6 +2006,11 @@
           <t>386</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1783,6 +2018,11 @@
           <t>387</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1790,6 +2030,11 @@
           <t>388</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3A, 3B, 4A, 4B, 5, 6, 7A1, 7A2, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1797,6 +2042,11 @@
           <t>389</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 2, 3, 4, 5A, 5B, 5C, 6, 7, 8A, 8B, 9A1A, 9A2, 9A3, 9A4, 9A5, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1804,6 +2054,11 @@
           <t>390</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 10E, 10F, 10G, 10H1, 10H2, 10I, 10J, 11, 12, 13, 14, 15, 16, 17, 2, 3A, 3B, 3C1, 3C2, 3C3, 3C4, 3C5, 3C6, 3C7, 3D1A, 3D2, 3D3, 3E1A1, 3E1B, 3E1C, 3E1D, 3E2, 3F1A, 3F1B, 3F2, 3F3, 3F4, 3G1A1, 3G1B, 3G1C, 3G2, 6C, 7A1, 7A2, 7B1A1, 7B1A2, 7B1B, 7B2, 7C, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1811,6 +2066,11 @@
           <t>391</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 2A, 2B, 3A1, 3A2, 3A3, 3B, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1818,6 +2078,11 @@
           <t>392</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4A, 4B, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1825,6 +2090,11 @@
           <t>393</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 1A, 1B, 2A1, 2A2, 2B, 3A, 3B, 4, 5, 6, 7, 8A, 8B1, 8B2, 8B3, 8B4, 9</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1832,6 +2102,11 @@
           <t>394</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1839,6 +2114,11 @@
           <t>395</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1846,6 +2126,11 @@
           <t>396</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1A4, 1B1, 1B2, 2A, 2B, 2C, 2D, 2E</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1853,6 +2138,11 @@
           <t>397</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -1860,6 +2150,11 @@
           <t>398</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -1867,6 +2162,11 @@
           <t>399</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5, 6A, 6B1, 6B2, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -1874,6 +2174,11 @@
           <t>400</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -1881,6 +2186,11 @@
           <t>401</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 2, 3, 4, 5, 6, 7, 8A1, 8A2, 8B1, 8B2, 9</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -1888,6 +2198,11 @@
           <t>402</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 3, 4, 5A1, 5B, 5C1, 5C2, 5C3, 6A, 6B, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -1895,6 +2210,11 @@
           <t>403</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2A, 2A2B, 2A3, 2A4, 2A5A, 2A5B1, 2A5B2, 2A6A, 2A6B, 2A6C, 2B1A, 2B1B, 2B2, 3, 4A1, 4A2, 4A3, 4A4, 4B1, 4B2, 5</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -1902,6 +2222,11 @@
           <t>404</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 11, 2A, 2B, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -1909,6 +2234,11 @@
           <t>405</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1, 2A1, 2A2A1, 2A2A2, 2A2B, 2A3A1, 2A3A2, 2A3B, 2B1A, 2B1B, 2B2, 2C, 2D1A, 2D1B, 2D2, 3, 4A, 4B, 5A, 5B, 6A, 6B, 7A1, 7A2, 7A3, 7A4</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -1916,6 +2246,11 @@
           <t>406</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>10A1A, 10A1B, 10A2, 10B1A1, 10B1A2, 10B1B, 10C1A, 10C1B, 10C2, 11A1, 11A2, 11B, 12, 13A, 13B, 14, 15, 16, 17, 18, 19A1A, 19A1B, 19A2, 19B1A, 19B1B, 19B2, 1A, 1B, 2A, 2B, 3A, 3B1A, 3B1B, 3B2, 4A, 4B1, 4B2, 4C1, 4C2, 5A1A, 5A1B, 5A2A, 5A2B, 5B, 6A, 6B, 7A1, 7A2, 7B, 8A1, 8A2, 8B1, 8B2, 9A, 9B1, 9B2, 9C1, 9C2</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -1923,6 +2258,11 @@
           <t>407</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C1, 1C2, 2, 3A1, 3A2, 3B, 3C, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -1930,6 +2270,11 @@
           <t>408</t>
         </is>
       </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 2, 3, 4, 5A, 5B, 6, 7A, 7B, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -1937,6 +2282,11 @@
           <t>409</t>
         </is>
       </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -1944,6 +2294,11 @@
           <t>410</t>
         </is>
       </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -1951,6 +2306,11 @@
           <t>411</t>
         </is>
       </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1, 10A1A, 10B1, 10C1, 11, 11A1A, 11A1B, 11B1A1, 11B1A2, 11B1B, 11B2, 12, 13, 14, 15, 16, 17, 18A, 19, 20, 21, 22, 23, 24A, 24B, 25, 26, 27, 28, 2A, 2B, 2C, 3A, 3B1, 3B2, 4A1, 4A2, 4B1, 4B2, 4C1, 4C2, 5A, 5B, 6, 7, 8, 9A, 9B1A1, 9B2, 9B3</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -1958,6 +2318,11 @@
           <t>412</t>
         </is>
       </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1A1A, 1A1B, 1A1C, 1A1D, 1A2, 1B, 2, 3, 4A, 4B, 5, 6A, 6B, 6C, 7, 8A1A, 8A1B, 8A2, 8B1A1, 8B1A2, 8B1B, 8C1A1, 8C1A2, 8C1B, 8C2A1A, 8C2A1B, 8C2B, 8D, 8E1, 8E2, 8F1A, 8F1B, 8F2, 9</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -1965,6 +2330,11 @@
           <t>413</t>
         </is>
       </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -1972,6 +2342,11 @@
           <t>414</t>
         </is>
       </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -1979,6 +2354,11 @@
           <t>415</t>
         </is>
       </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5A, 5B, 6A, 6B, 7A1, 7A2, 7B1, 7B2</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -1986,6 +2366,11 @@
           <t>416</t>
         </is>
       </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -1993,6 +2378,11 @@
           <t>417</t>
         </is>
       </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2A, 2B, 3, 4, 5A, 5B, 5C, 5D, 5E, 5F, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -2000,6 +2390,11 @@
           <t>418</t>
         </is>
       </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 2, 3, 4, 5, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -2007,6 +2402,11 @@
           <t>419</t>
         </is>
       </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -2014,6 +2414,11 @@
           <t>420</t>
         </is>
       </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -2021,6 +2426,11 @@
           <t>421</t>
         </is>
       </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2, 3, 4, 5A, 5B, 6A, 6B1, 6B2, 6C, 7</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -2028,6 +2438,11 @@
           <t>422</t>
         </is>
       </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1A, 1B1A, 1B1B1, 1B1B2, 2A1, 2A2, 3A, 3B, 4A, 4B, 5, 6A1A, 6A1B, 6A2, 6B1, 6B2A1, 6B2A2, 6B2B, 6B3, 6B4, 6B5A, 6B5B</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -2035,6 +2450,11 @@
           <t>423</t>
         </is>
       </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7A, 7B, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -2042,6 +2462,11 @@
           <t>424</t>
         </is>
       </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -2049,6 +2474,11 @@
           <t>425</t>
         </is>
       </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1A1A1, 1A1A2, 1A1B, 1A2, 1B1, 1B3, 2, 3A, 3B, 4, 5, 6, 7A, 7B, 8A1A, 8A1B, 8A2, 8B1, 8B2, 9</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -2056,6 +2486,11 @@
           <t>426</t>
         </is>
       </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -2063,6 +2498,11 @@
           <t>427</t>
         </is>
       </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -2070,11 +2510,21 @@
           <t>428</t>
         </is>
       </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3A, 1A3C, 1A4A, 1A4B, 1A5, 1A6, 1A7, 1A8, 1A9, 1B1A, 1B1B, 1B2, 1C1A, 1C1B, 1C2, 2A1A, 2A1B, 2A1C, 2A2, 2A3, 2A4, 2B, 2C</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
           <t>429</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 5A, 5B, 6A1A, 6A1B, 6A2, 6B, 7, 8A, 8B1, 8B2, 9A, 9B, 9C</t>
         </is>
       </c>
     </row>

</xml_diff>